<commit_message>
yearbook: add per-capita GDP, inward FDI & outward ODI (national + by-country)
- 人均地区生产总值 (provincial per-capita GDP) from table 3-9
- Inward FDI: 11-13 national time series + 11-14 by source country/region
- Outward ODI: 11-18 national time series + 11-19 by destination country/region
- Fix per-capita column index and drop title rows in country tables

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GrCg46UpnRBrGiga5w9ZJC
</commit_message>
<xml_diff>
--- a/output/china_yearbook_provincial.xlsx
+++ b/output/china_yearbook_provincial.xlsx
@@ -9,11 +9,16 @@
   <sheets>
     <sheet name="説明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="GDP 地区生产总值" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="小売 社会消费品零售总额" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="貿易 货物进出口" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="不動産 开发完成投资" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="全国 商品房销售面积" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="全国 商品房销售额" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="一人当たりGDP 人均" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="小売 社会消费品零售总额" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="貿易 货物进出口" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="不動産 开发完成投资" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="全国 商品房销售面积" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="全国 商品房销售额" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="対中投資FDI(全国推移)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="対外投資ODI(全国推移)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="対中投資FDI(国別)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="対外投資ODI(国別)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +31,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +46,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -77,6 +86,8 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,6 +509,2535 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>対外投資ODI(全国推移)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>単位: 億米ドル / 100 mil. USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>年 / Year</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>122.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>211.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>265.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>559.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>565.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>688.1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>746.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>1078.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1231.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>1456.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>1961.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>1582.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>1430.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>1369.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>1537.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>1788.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2006-2021年为全行业对外直接投资数据。</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C129"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>対中投資FDI(国別)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>単位: 万米ドル / 10,000 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>国・地域 / Country</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>总计</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>18095721</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>18913241</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>亚洲</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>15364464</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>16356555</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>孟加拉国</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>文莱</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>658</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>缅甸</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>柬埔寨</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>3369</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>5217</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>塞浦路斯</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>460</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>15075</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>中国香港</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>13175642</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>13724149</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>632</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>印度尼西亚</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>2434</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>伊拉克</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>4255</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>8101</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>391325</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>460508</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>约旦</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>344</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>科威特</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>192</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>老挝</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>黎巴嫩</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>中国澳门</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>218948</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>124291</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>马来西亚</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>5770</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>112697</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>蒙古</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>506</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>巴基斯坦</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>941</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>卡塔尔</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>沙特阿拉伯</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>7300</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>7898</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>新加坡</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>1033164</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>1059894</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>韩国</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>404469</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>659872</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>斯里兰卡</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>泰国</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>10741</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>6809</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>5243</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>阿联酋</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>2229</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>96424</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>也门</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>越南</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>603</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>中国台湾</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>93990</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>66110</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>东帝汶</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>土库曼斯坦</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>乌兹别克斯坦</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>483</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>108884</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>33765</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>喀麦隆</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>501</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>刚果(布)</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>埃及</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>埃塞俄比亚</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>加纳</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>马里</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>毛里塔尼亚</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>396</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>毛里求斯</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>89774</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>6594</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>摩洛哥</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>纳米比亚</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n">
+        <v>853</v>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>塞舌尔</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>16868</v>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>14572</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>南非</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="n">
+        <v>384</v>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>10319</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>坦桑尼亚</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>乌干达</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>赞比亚</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>非洲其他国家(地区)</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="n">
+        <v>77</v>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="n">
+        <v>711570</v>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>1197604</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="n">
+        <v>11519</v>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>18353</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="n">
+        <v>21713</v>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>42596</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n">
+        <v>119971</v>
+      </c>
+      <c r="C61" s="7" t="n">
+        <v>159819</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>168019</v>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>256643</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="n">
+        <v>71013</v>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>75650</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="n">
+        <v>19341</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>17095</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="n">
+        <v>17756</v>
+      </c>
+      <c r="C65" s="7" t="n">
+        <v>14847</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>卢森堡</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="n">
+        <v>31091</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <v>16059</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="n">
+        <v>110544</v>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>449402</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="n">
+        <v>720</v>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="n">
+        <v>8936</v>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>12335</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>安道尔</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="n">
+        <v>9368</v>
+      </c>
+      <c r="C72" s="7" t="n">
+        <v>15530</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="n">
+        <v>6333</v>
+      </c>
+      <c r="C74" s="7" t="n">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="n">
+        <v>720</v>
+      </c>
+      <c r="C75" s="7" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>冰岛</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="n">
+        <v>79</v>
+      </c>
+      <c r="C76" s="7" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>列支敦士登</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="n">
+        <v>1077</v>
+      </c>
+      <c r="C77" s="7" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>摩纳哥</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="n">
+        <v>260</v>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="n">
+        <v>5559</v>
+      </c>
+      <c r="C79" s="7" t="n">
+        <v>6623</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>444</v>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="n">
+        <v>202</v>
+      </c>
+      <c r="C81" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="n">
+        <v>30141</v>
+      </c>
+      <c r="C82" s="7" t="n">
+        <v>54233</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="n">
+        <v>73144</v>
+      </c>
+      <c r="C83" s="7" t="n">
+        <v>39152</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C84" s="7" t="n">
+        <v>10111</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="C85" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>阿塞拜疆</t>
+        </is>
+      </c>
+      <c r="B86" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C86" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>白俄罗斯</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C87" s="7" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>俄罗斯联邦</t>
+        </is>
+      </c>
+      <c r="B88" s="7" t="n">
+        <v>754</v>
+      </c>
+      <c r="C88" s="7" t="n">
+        <v>3895</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C90" s="7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="n">
+        <v>408</v>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="7" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>欧洲其他国家(地区)</t>
+        </is>
+      </c>
+      <c r="B94" s="7" t="n">
+        <v>1255</v>
+      </c>
+      <c r="C94" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>拉丁美洲</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="n">
+        <v>783725</v>
+      </c>
+      <c r="C95" s="7" t="n">
+        <v>916876</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>安提瓜和巴布达</t>
+        </is>
+      </c>
+      <c r="B96" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" s="7" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>阿根廷</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>巴巴多斯</t>
+        </is>
+      </c>
+      <c r="B98" s="7" t="n">
+        <v>1353</v>
+      </c>
+      <c r="C98" s="7" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>伯利兹</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="n">
+        <v>2538</v>
+      </c>
+      <c r="C99" s="7" t="n">
+        <v>3450</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="n">
+        <v>1553</v>
+      </c>
+      <c r="C100" s="7" t="n">
+        <v>2581</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>开曼群岛</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="n">
+        <v>246157</v>
+      </c>
+      <c r="C101" s="7" t="n">
+        <v>241631</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>智利</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="n">
+        <v>427</v>
+      </c>
+      <c r="C102" s="7" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>古巴</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="C103" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>多米尼加共和国</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>危地马拉</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="C105" s="7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>圭亚那</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C106" s="7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>墨西哥</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="n">
+        <v>373</v>
+      </c>
+      <c r="C107" s="7" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>巴拿马</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="n">
+        <v>144</v>
+      </c>
+      <c r="C108" s="7" t="n">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>秘鲁</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="C109" s="7" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>特立尼达和多巴哥</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>特克斯和凯科斯群岛</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" s="7" t="n">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>乌拉圭</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C112" s="7" t="n">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>委内瑞拉</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C113" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>英属维尔京群岛</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="n">
+        <v>528097</v>
+      </c>
+      <c r="C114" s="7" t="n">
+        <v>663493</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>圣其茨和尼维斯</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="n">
+        <v>725</v>
+      </c>
+      <c r="C115" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>拉丁美洲其他国家(地区)</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="n">
+        <v>2137</v>
+      </c>
+      <c r="C116" s="7" t="n">
+        <v>2401</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>北美洲</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="n">
+        <v>279199</v>
+      </c>
+      <c r="C117" s="7" t="n">
+        <v>287839</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="n">
+        <v>20269</v>
+      </c>
+      <c r="C118" s="7" t="n">
+        <v>16571</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="n">
+        <v>246746</v>
+      </c>
+      <c r="C119" s="7" t="n">
+        <v>221457</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>百慕大</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="n">
+        <v>12184</v>
+      </c>
+      <c r="C120" s="7" t="n">
+        <v>49811</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>大洋洲</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="n">
+        <v>98004</v>
+      </c>
+      <c r="C121" s="7" t="n">
+        <v>120516</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="n">
+        <v>29953</v>
+      </c>
+      <c r="C122" s="7" t="n">
+        <v>40211</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>库克群岛</t>
+        </is>
+      </c>
+      <c r="B123" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C123" s="7" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>新西兰</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="n">
+        <v>1782</v>
+      </c>
+      <c r="C124" s="7" t="n">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>萨摩亚</t>
+        </is>
+      </c>
+      <c r="B125" s="7" t="n">
+        <v>62144</v>
+      </c>
+      <c r="C125" s="7" t="n">
+        <v>74734</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>马绍尔群岛</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="n">
+        <v>2705</v>
+      </c>
+      <c r="C126" s="7" t="n">
+        <v>4271</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>大洋洲其他国家(地区)</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="n">
+        <v>1420</v>
+      </c>
+      <c r="C127" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="n">
+        <v>2485</v>
+      </c>
+      <c r="C128" s="7" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>注：2021年各国家(地区)数据不包含银行、证券、保险领域数据。</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="n">
+        <v/>
+      </c>
+      <c r="C129" s="7" t="n">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>対外投資ODI(国別)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>単位: 万米ドル / 10,000 USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>国・地域 / Country</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2020流量</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2021流量</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2021末存量</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>15371026</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>17881932</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>278514971</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>亚洲</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>11234365</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>12810205</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>177201520</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>中国香港</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>8914586</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>10119088</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>154965764</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>20519</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>27946</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>351889</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>印度尼西亚</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>219835</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>437251</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>2008048</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>48683</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>76214</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>488287</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>中国澳门</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>82684</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>88192</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1123624</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>新加坡</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>592335</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>840504</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>6720228</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>韩国</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>13914</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>47804</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>660150</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>泰国</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>188288</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>148601</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>991721</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>越南</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>187575</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>220762</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>1085211</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>422560</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>498664</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>4418621</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>阿尔及利亚</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>1864</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>18471</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>171602</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>苏丹</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>283</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>9429</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>111552</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>几内亚</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>-29512</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>48717</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>95933</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>马达加斯加</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>13598</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>-962</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>32287</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>尼日利亚</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>30894</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>20167</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>269579</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>南非</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>40043</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>36359</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>529417</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>1269565</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>1087480</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>13479438</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>92222</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>190355</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>1900531</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>137560</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>271113</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>1669749</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>14779</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>-15167</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>486390</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>俄罗斯联邦</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>57032</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>-107230</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>1064411</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>拉丁美洲</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>1665651</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>2615851</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>69374017</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>31264</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>14645</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>300771</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>开曼群岛</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>856222</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>1075356</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>22952507</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>墨西哥</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>26456</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>23183</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>130216</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>英属维尔京群岛</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>697562</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>1397101</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>44747734</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>北美洲</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>634312</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>658090</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>10022580</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>21002</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>93017</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>1379315</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>601867</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>558435</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>7717236</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>大洋洲</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>144573</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>211642</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>4018796</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>119859</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>192254</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>3443047</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>新西兰</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>45292</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>22461</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>312871</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -947,6 +3487,354 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>一人当たりGDP 人均</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>地区/地域</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>人均地区生产总值(元)
+2022 値</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>190313</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>119235</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>河北</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>56995</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>山西</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>73675</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>内モンゴル</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>96474</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>遼寧</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>68775</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>吉林</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>55347</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>黒龍江</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>51096</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>179907</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>江蘇</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>144390</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>浙江</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>118496</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>安徽</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>73603</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>福建</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>126829</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>江西</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>70923</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>山東</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>86003</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>河南</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>62106</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>湖北</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>92059</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>湖南</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>73598</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>広東</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>101905</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>広西</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>52164</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>海南</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>66602</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>重慶</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>90663</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>四川</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>67777</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>貴州</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>52321</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>雲南</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>61716</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>チベット</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>58438</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>陝西</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>82864</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>甘粛</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>44968</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>青海</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>60724</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>寧夏</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>69781</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>新疆</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>68552</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1613,7 +4501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2177,7 +5065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2447,244 +5335,6 @@
       </c>
       <c r="B35" s="4" t="n">
         <v>1158.8633</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>全国 商品房销售面积</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>地区/地域</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-1998 値</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2000 値</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2005 値</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2006 値</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2007 値</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2008 値</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2009 値</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2010 値</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2011 値</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2012 値</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2013 値</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2014 値</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2015 値</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2016 値</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2017 値</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2018 値</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2019 値</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2020 値</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2021 値</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>商品房销售面积
-2022 値</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>全国</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>12185.3</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>18637.128</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>55486.2247</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>61857.0733</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>77354.71799999999</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>65969.83</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>94755</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>104482.7556101567</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>108662.065834563</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>110074.6726904123</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>128347.0683570207</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>118335.9970251731</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>125475.7646102896</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>152578.5297661122</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>163427.0326061051</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>164947.3403961267</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>164531.4239690406</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>168560.4128347682</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>171414.5985785524</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>129766.3947</v>
       </c>
     </row>
   </sheetData>
@@ -2727,7 +5377,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>全国 商品房销售额</t>
+          <t>全国 商品房销售面积</t>
         </is>
       </c>
     </row>
@@ -2739,6 +5389,244 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>商品房销售面积
+1998 値</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2000 値</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2005 値</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2006 値</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2007 値</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2008 値</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2009 値</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2010 値</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2011 値</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2012 値</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2013 値</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2014 値</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2015 値</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2016 値</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2017 値</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2018 値</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2019 値</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2020 値</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2021 値</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>商品房销售面积
+2022 値</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>12185.3</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>18637.128</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>55486.2247</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>61857.0733</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>77354.71799999999</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>65969.83</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>94755</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>104482.7556101567</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>108662.065834563</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>110074.6726904123</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>128347.0683570207</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>118335.9970251731</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>125475.7646102896</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>152578.5297661122</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>163427.0326061051</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>164947.3403961267</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>164531.4239690406</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>168560.4128347682</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>171414.5985785524</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>129766.3947</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>全国 商品房销售额</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>地区/地域</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>商品房销售额
 1998 値</t>
         </is>
@@ -2923,6 +5811,460 @@
       </c>
       <c r="U4" s="4" t="n">
         <v>129655.5699</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>対中投資FDI(全国推移)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>単位: 億米ドル / 100 mil. USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>年 / Year</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>金額</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1979-1982</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1983</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1985</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>19.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1986</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>22.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1987</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>31.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>33.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1991</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>43.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>110.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>275.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>337.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>375.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>417.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>452.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>454.6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>403.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>407.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>468.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2002</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>527.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>606.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>724.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>727.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>835.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>1083.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>940.6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>1147.3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>1239.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>1210.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>1239.1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>1355.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>1337.1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>1363.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>1383.1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>1412.2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>1493.4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>1809.6</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>1891.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>